<commit_message>
ingesta: snapshot 2026-07-12 18:09 UTC
</commit_message>
<xml_diff>
--- a/data_lake/datos_diarios_preliminares/dt=2026-07-12/CORDOBA_JUL26.xlsx
+++ b/data_lake/datos_diarios_preliminares/dt=2026-07-12/CORDOBA_JUL26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Mi unidad\OSPA\02. Datos Diarios\Tablas\Datos hidrometeorologicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EFA47D9-5C33-4EEF-BACD-37DC2BAA49A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B90D408-1AEF-45D4-A44A-D7A7EE507FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{5F8F14AC-D557-4126-B18A-7A2C1E69122F}"/>
   </bookViews>
@@ -9990,7 +9990,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-1</c:v>
+                  <c:v>19.399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>-1</c:v>
@@ -19949,7 +19949,9 @@
       <c r="N3" s="25">
         <v>0</v>
       </c>
-      <c r="O3" s="25"/>
+      <c r="O3" s="25">
+        <v>0</v>
+      </c>
       <c r="P3" s="25"/>
       <c r="Q3" s="25"/>
       <c r="R3" s="25"/>
@@ -20021,7 +20023,9 @@
       <c r="N4" s="25">
         <v>0</v>
       </c>
-      <c r="O4" s="25"/>
+      <c r="O4" s="25">
+        <v>0</v>
+      </c>
       <c r="P4" s="25"/>
       <c r="Q4" s="25"/>
       <c r="R4" s="25"/>
@@ -20093,7 +20097,9 @@
       <c r="N5" s="25">
         <v>0</v>
       </c>
-      <c r="O5" s="25"/>
+      <c r="O5" s="25">
+        <v>2</v>
+      </c>
       <c r="P5" s="25"/>
       <c r="Q5" s="25"/>
       <c r="R5" s="25"/>
@@ -20116,7 +20122,7 @@
       <c r="AI5" s="34"/>
       <c r="AJ5" s="36">
         <f t="shared" si="0"/>
-        <v>44.1</v>
+        <v>46.1</v>
       </c>
       <c r="AK5" s="30">
         <v>40.986206896551728</v>
@@ -20165,7 +20171,9 @@
       <c r="N6" s="25">
         <v>0</v>
       </c>
-      <c r="O6" s="25"/>
+      <c r="O6" s="25">
+        <v>17.399999999999999</v>
+      </c>
       <c r="P6" s="25"/>
       <c r="Q6" s="25"/>
       <c r="R6" s="25"/>
@@ -20188,7 +20196,7 @@
       <c r="AI6" s="34"/>
       <c r="AJ6" s="36">
         <f t="shared" si="0"/>
-        <v>83.100000000000009</v>
+        <v>100.5</v>
       </c>
       <c r="AK6" s="30">
         <v>88.719230769230762</v>
@@ -20341,7 +20349,9 @@
       <c r="N9" s="25">
         <v>0</v>
       </c>
-      <c r="O9" s="25"/>
+      <c r="O9" s="25">
+        <v>0</v>
+      </c>
       <c r="P9" s="25"/>
       <c r="Q9" s="25"/>
       <c r="R9" s="25"/>
@@ -20413,7 +20423,9 @@
       <c r="N10" s="25">
         <v>0</v>
       </c>
-      <c r="O10" s="25"/>
+      <c r="O10" s="25">
+        <v>0</v>
+      </c>
       <c r="P10" s="25"/>
       <c r="Q10" s="25"/>
       <c r="R10" s="25"/>
@@ -20483,7 +20495,9 @@
       <c r="N11" s="25">
         <v>0</v>
       </c>
-      <c r="O11" s="25"/>
+      <c r="O11" s="25">
+        <v>0</v>
+      </c>
       <c r="P11" s="25"/>
       <c r="Q11" s="25"/>
       <c r="R11" s="25"/>
@@ -20551,7 +20565,9 @@
       <c r="N12" s="25">
         <v>0</v>
       </c>
-      <c r="O12" s="25"/>
+      <c r="O12" s="25">
+        <v>0</v>
+      </c>
       <c r="P12" s="25"/>
       <c r="Q12" s="25"/>
       <c r="R12" s="25"/>
@@ -20693,7 +20709,9 @@
       <c r="N14" s="25">
         <v>0</v>
       </c>
-      <c r="O14" s="25"/>
+      <c r="O14" s="25">
+        <v>0</v>
+      </c>
       <c r="P14" s="25"/>
       <c r="Q14" s="25"/>
       <c r="R14" s="25"/>
@@ -20765,7 +20783,9 @@
       <c r="N15" s="25">
         <v>0</v>
       </c>
-      <c r="O15" s="25"/>
+      <c r="O15" s="25">
+        <v>0</v>
+      </c>
       <c r="P15" s="25"/>
       <c r="Q15" s="25"/>
       <c r="R15" s="25"/>
@@ -20938,7 +20958,7 @@
       </c>
       <c r="O19" s="26">
         <f t="shared" si="1"/>
-        <v>-1</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="P19" s="26">
         <f t="shared" si="1"/>

</xml_diff>